<commit_message>
Fix: Carga completa de 250 paises desde JSON mirror
</commit_message>
<xml_diff>
--- a/src/xlsx/ingestion.xlsx
+++ b/src/xlsx/ingestion.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,6 +470,1786 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ABW</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Aruba</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Aruba</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Oranjestad</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Caribbean</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AFG</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Afghanistan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Islamic Republic of Afghanistan</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Kabul</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Southern Asia</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>652230</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AGO</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Angola</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Republic of Angola</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Middle Africa</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>1246700</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AIA</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Anguilla</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Anguilla</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>The Valley</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Caribbean</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ALA</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Åland Islands</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Åland Islands</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Mariehamn</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Northern Europe</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>1580</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ALB</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Albania</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Republic of Albania</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Tirana</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Southeast Europe</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>28748</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AND</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Andorra</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Principality of Andorra</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Andorra la Vella</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Southern Europe</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ARE</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Abu Dhabi</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Western Asia</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>83600</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ARG</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Argentine Republic</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>South America</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>2780400</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Armenia</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Republic of Armenia</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Yerevan</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Western Asia</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>29743</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ASM</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>American Samoa</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>American Samoa</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Pago Pago</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Oceania</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Polynesia</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ATA</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Antarctica</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Antarctica</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Antarctic</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>14000000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ATF</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>French Southern and Antarctic Lands</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Territory of the French Southern and Antarctic Lands</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Port-aux-Français</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Antarctic</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>7747</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ATG</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Antigua and Barbuda</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Antigua and Barbuda</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Saint John's</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Caribbean</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AUS</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Commonwealth of Australia</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Canberra</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Oceania</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Australia and New Zealand</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>7692024</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AUT</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Republic of Austria</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Vienna</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Central Europe</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>83871</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AZE</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Republic of Azerbaijan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Baku</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Western Asia</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BDI</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Burundi</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Republic of Burundi</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Gitega</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Eastern Africa</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>27834</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Kingdom of Belgium</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Brussels</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Western Europe</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>30528</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BEN</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Benin</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Republic of Benin</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Porto-Novo</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Western Africa</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>112622</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BFA</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Ouagadougou</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Western Africa</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>272967</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BGD</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>People's Republic of Bangladesh</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Dhaka</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Southern Asia</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>147570</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BGR</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Republic of Bulgaria</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Southeast Europe</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>110879</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BHR</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Bahrain</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Kingdom of Bahrain</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Manama</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Western Asia</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BHS</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Bahamas</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Commonwealth of the Bahamas</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Nassau</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Caribbean</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>13943</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>BIH</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Bosnia and Herzegovina</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Bosnia and Herzegovina</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Sarajevo</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Southeast Europe</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>51209</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BLM</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Saint Barthélemy</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Collectivity of Saint Barthélemy</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Gustavia</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Caribbean</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SHN</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Saint Helena, Ascension and Tristan da Cunha</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Saint Helena, Ascension and Tristan da Cunha</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Jamestown</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Western Africa</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BLR</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Belarus</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Republic of Belarus</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Minsk</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Eastern Europe</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="n">
+        <v>207600</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BLZ</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Belize</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Belize</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Belmopan</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Central America</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="n">
+        <v>22966</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BMU</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Hamilton</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>BOL</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Bolivia</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Plurinational State of Bolivia</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>South America</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="n">
+        <v>1098581</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BES</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Caribbean Netherlands</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Bonaire, Sint Eustatius and Saba</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Kralendijk</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Caribbean</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="n">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>BRA</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Federative Republic of Brazil</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>South America</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="n">
+        <v>8515767</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>BRB</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Barbados</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Barbados</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Bridgetown</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Caribbean</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>BRN</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Brunei</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Nation of Brunei, Abode of Peace</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Bandar Seri Begawan</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>South-Eastern Asia</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="n">
+        <v>5765</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BTN</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Bhutan</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Kingdom of Bhutan</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Thimphu</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Southern Asia</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="n">
+        <v>38394</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>BVT</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Bouvet Island</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Bouvet Island</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Antarctic</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BWA</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Republic of Botswana</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Gaborone</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Southern Africa</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="n">
+        <v>582000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CAF</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Central African Republic</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Central African Republic</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Bangui</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Middle Africa</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="n">
+        <v>622984</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>CAN</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="n">
+        <v>9984670</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>CCK</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Cocos (Keeling) Islands</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Territory of the Cocos (Keeling) Islands</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>West Island</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Oceania</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Australia and New Zealand</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CHE</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Swiss Confederation</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Bern</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Western Europe</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="n">
+        <v>41284</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>CHL</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Republic of Chile</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Santiago</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>South America</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="n">
+        <v>756102</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>CHN</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>People's Republic of China</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Beijing</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Eastern Asia</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="n">
+        <v>9706961</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>CIV</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Ivory Coast</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Republic of Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Yamoussoukro</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Western Africa</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="n">
+        <v>322463</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>CMR</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Cameroon</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Republic of Cameroon</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Yaoundé</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Middle Africa</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="n">
+        <v>475442</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>DR Congo</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Democratic Republic of the Congo</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Kinshasa</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Middle Africa</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="n">
+        <v>2344858</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>COG</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Congo</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Republic of the Congo</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Brazzaville</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Middle Africa</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="n">
+        <v>342000</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>COK</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Cook Islands</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Cook Islands</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Avarua</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Oceania</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Polynesia</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="n">
+        <v>236</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>